<commit_message>
Phase 3-B WS2 deploy: S1 prior-signal state + D1 confidence damping (era A-S1D1)
Two-channel logging: confidence_raw on every line (raw = model channel, operative = system truth). Phase-agnostic ACCOUNT_RE in the tracker parser (3-B cutover bug caught pre-deploy). h1_lag_trace: --raw-from-logs (AM-canonical) + --suffix. Weekly runner: GM tracer, post-deploy two-channel acceptance slices, --stratify-regime (T2 sensor). New: signal_state.py + seed_signal_state.py. README to 3-B; spec + deploy notes in docs/.
</commit_message>
<xml_diff>
--- a/tracker_with_registry.xlsx
+++ b/tracker_with_registry.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rober\claude-equity-bot\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8822953C-CF5D-458B-8041-D437EE37D391}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D3175F2-2ACA-4153-BD82-439C50CF466D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" firstSheet="1" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3618" uniqueCount="348">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3714" uniqueCount="348">
   <si>
     <t>Live Cohort Scoreboard — Phase 3-A out-of-sample guardrail</t>
   </si>
@@ -1658,30 +1658,30 @@
     <xf numFmtId="0" fontId="0" fillId="15" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2012,31 +2012,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="96" t="s">
+      <c r="A1" s="99" t="s">
         <v>34</v>
       </c>
-      <c r="B1" s="93"/>
-      <c r="C1" s="93"/>
-      <c r="D1" s="93"/>
-      <c r="E1" s="93"/>
+      <c r="B1" s="97"/>
+      <c r="C1" s="97"/>
+      <c r="D1" s="97"/>
+      <c r="E1" s="97"/>
     </row>
     <row r="2" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="94" t="s">
+      <c r="A2" s="96" t="s">
         <v>35</v>
       </c>
-      <c r="B2" s="93"/>
-      <c r="C2" s="93"/>
-      <c r="D2" s="93"/>
-      <c r="E2" s="93"/>
+      <c r="B2" s="97"/>
+      <c r="C2" s="97"/>
+      <c r="D2" s="97"/>
+      <c r="E2" s="97"/>
     </row>
     <row r="4" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="95" t="s">
+      <c r="A4" s="98" t="s">
         <v>36</v>
       </c>
-      <c r="B4" s="93"/>
-      <c r="C4" s="93"/>
-      <c r="D4" s="93"/>
-      <c r="E4" s="93"/>
+      <c r="B4" s="97"/>
+      <c r="C4" s="97"/>
+      <c r="D4" s="97"/>
+      <c r="E4" s="97"/>
     </row>
     <row r="5" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
@@ -2044,7 +2044,7 @@
       </c>
       <c r="B5" s="4">
         <f>COUNTA(Signals!B5:B2000)</f>
-        <v>787</v>
+        <v>811</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2071,7 +2071,7 @@
       </c>
       <c r="B8" s="4">
         <f>COUNTIF(Signals!D5:D2000,"HOLD")</f>
-        <v>764</v>
+        <v>788</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2080,17 +2080,17 @@
       </c>
       <c r="B9" s="5">
         <f>COUNTIF(Signals!D5:D2000,"HOLD")/COUNTA(Signals!D5:D2000)</f>
-        <v>0.97324840764331211</v>
+        <v>0.97404202719406674</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="95" t="s">
+      <c r="A11" s="98" t="s">
         <v>42</v>
       </c>
-      <c r="B11" s="93"/>
-      <c r="C11" s="93"/>
-      <c r="D11" s="93"/>
-      <c r="E11" s="93"/>
+      <c r="B11" s="97"/>
+      <c r="C11" s="97"/>
+      <c r="D11" s="97"/>
+      <c r="E11" s="97"/>
     </row>
     <row r="12" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
@@ -2098,7 +2098,7 @@
       </c>
       <c r="B12" s="5">
         <f>AVERAGE(Signals!E5:E2000)</f>
-        <v>0.52991082802547784</v>
+        <v>0.5299258343634119</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2143,7 +2143,7 @@
       </c>
       <c r="B17" s="6">
         <f>COUNTIF(Signals!E5:E2000,"&gt;=0.6")</f>
-        <v>182</v>
+        <v>190</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2152,7 +2152,7 @@
       </c>
       <c r="B18" s="6">
         <f>COUNTIF(Signals!E5:E2000,"&lt;0.45")</f>
-        <v>135</v>
+        <v>139</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2161,17 +2161,17 @@
       </c>
       <c r="B19" s="6">
         <f>COUNTIF(Signals!E5:E2000,"&lt;0.40")</f>
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="95" t="s">
+      <c r="A22" s="98" t="s">
         <v>51</v>
       </c>
-      <c r="B22" s="93"/>
-      <c r="C22" s="93"/>
-      <c r="D22" s="93"/>
-      <c r="E22" s="93"/>
+      <c r="B22" s="97"/>
+      <c r="C22" s="97"/>
+      <c r="D22" s="97"/>
+      <c r="E22" s="97"/>
     </row>
     <row r="23" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="7" t="s">
@@ -2190,11 +2190,11 @@
       </c>
       <c r="B24" s="4">
         <f>COUNTIF(Signals!F5:F2000,"HIGH")</f>
-        <v>344</v>
+        <v>362</v>
       </c>
       <c r="C24" s="5">
         <f>B24/SUM(B24:B26)</f>
-        <v>0.43821656050955415</v>
+        <v>0.44746600741656367</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2203,11 +2203,11 @@
       </c>
       <c r="B25" s="4">
         <f>COUNTIF(Signals!F5:F2000,"MEDIUM")</f>
-        <v>420</v>
+        <v>426</v>
       </c>
       <c r="C25" s="5">
         <f>B25/SUM(B24:B26)</f>
-        <v>0.53503184713375795</v>
+        <v>0.52657601977750312</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2220,26 +2220,26 @@
       </c>
       <c r="C26" s="5">
         <f>B26/SUM(B24:B26)</f>
-        <v>2.6751592356687899E-2</v>
+        <v>2.595797280593325E-2</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="95" t="s">
+      <c r="A29" s="98" t="s">
         <v>58</v>
       </c>
-      <c r="B29" s="93"/>
-      <c r="C29" s="93"/>
-      <c r="D29" s="93"/>
-      <c r="E29" s="93"/>
+      <c r="B29" s="97"/>
+      <c r="C29" s="97"/>
+      <c r="D29" s="97"/>
+      <c r="E29" s="97"/>
     </row>
     <row r="30" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="94" t="s">
+      <c r="A30" s="96" t="s">
         <v>59</v>
       </c>
-      <c r="B30" s="93"/>
-      <c r="C30" s="93"/>
-      <c r="D30" s="93"/>
-      <c r="E30" s="93"/>
+      <c r="B30" s="97"/>
+      <c r="C30" s="97"/>
+      <c r="D30" s="97"/>
+      <c r="E30" s="97"/>
     </row>
     <row r="31" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="7" t="s">
@@ -2264,7 +2264,7 @@
       </c>
       <c r="B32" s="9">
         <f>COUNTIFS(Signals!E5:E2000,"&lt;0.4",Signals!E5:E2000,"&lt;0.4")</f>
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C32" s="9">
         <f>COUNTIFS(Signals!E5:E2000,"&lt;0.4",Signals!E5:E2000,"&lt;0.4",Signals!N5:N2000,"YES")</f>
@@ -2285,7 +2285,7 @@
       </c>
       <c r="B33" s="9">
         <f>COUNTIFS(Signals!E5:E2000,"&gt;=0.4",Signals!E5:E2000,"&lt;0.5")</f>
-        <v>210</v>
+        <v>217</v>
       </c>
       <c r="C33" s="9">
         <f>COUNTIFS(Signals!E5:E2000,"&gt;=0.4",Signals!E5:E2000,"&lt;0.5",Signals!N5:N2000,"YES")</f>
@@ -2306,7 +2306,7 @@
       </c>
       <c r="B34" s="9">
         <f>COUNTIFS(Signals!E5:E2000,"&gt;=0.5",Signals!E5:E2000,"&lt;0.6")</f>
-        <v>368</v>
+        <v>375</v>
       </c>
       <c r="C34" s="9">
         <f>COUNTIFS(Signals!E5:E2000,"&gt;=0.5",Signals!E5:E2000,"&lt;0.6",Signals!N5:N2000,"YES")</f>
@@ -2327,7 +2327,7 @@
       </c>
       <c r="B35" s="9">
         <f>COUNTIFS(Signals!E5:E2000,"&gt;=0.6",Signals!E5:E2000,"&lt;0.7")</f>
-        <v>181</v>
+        <v>189</v>
       </c>
       <c r="C35" s="9">
         <f>COUNTIFS(Signals!E5:E2000,"&gt;=0.6",Signals!E5:E2000,"&lt;0.7",Signals!N5:N2000,"YES")</f>
@@ -2385,13 +2385,13 @@
       </c>
     </row>
     <row r="40" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="95" t="s">
+      <c r="A40" s="98" t="s">
         <v>69</v>
       </c>
-      <c r="B40" s="93"/>
-      <c r="C40" s="93"/>
-      <c r="D40" s="93"/>
-      <c r="E40" s="93"/>
+      <c r="B40" s="97"/>
+      <c r="C40" s="97"/>
+      <c r="D40" s="97"/>
+      <c r="E40" s="97"/>
     </row>
     <row r="41" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="7" t="s">
@@ -2416,7 +2416,7 @@
       </c>
       <c r="B42" s="9">
         <f>COUNTIF(Signals!F5:F2000,"HIGH")</f>
-        <v>344</v>
+        <v>362</v>
       </c>
       <c r="C42" s="9">
         <f>COUNTIFS(Signals!F5:F2000,"HIGH",Signals!N5:N2000,"YES")</f>
@@ -2437,7 +2437,7 @@
       </c>
       <c r="B43" s="9">
         <f>COUNTIF(Signals!F5:F2000,"MEDIUM")</f>
-        <v>420</v>
+        <v>426</v>
       </c>
       <c r="C43" s="9">
         <f>COUNTIFS(Signals!F5:F2000,"MEDIUM",Signals!N5:N2000,"YES")</f>
@@ -2474,22 +2474,22 @@
       </c>
     </row>
     <row r="47" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="95" t="s">
+      <c r="A47" s="98" t="s">
         <v>72</v>
       </c>
-      <c r="B47" s="93"/>
-      <c r="C47" s="93"/>
-      <c r="D47" s="93"/>
-      <c r="E47" s="93"/>
+      <c r="B47" s="97"/>
+      <c r="C47" s="97"/>
+      <c r="D47" s="97"/>
+      <c r="E47" s="97"/>
     </row>
     <row r="48" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="94" t="s">
+      <c r="A48" s="96" t="s">
         <v>73</v>
       </c>
-      <c r="B48" s="93"/>
-      <c r="C48" s="93"/>
-      <c r="D48" s="93"/>
-      <c r="E48" s="93"/>
+      <c r="B48" s="97"/>
+      <c r="C48" s="97"/>
+      <c r="D48" s="97"/>
+      <c r="E48" s="97"/>
     </row>
     <row r="49" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="3" t="s">
@@ -2497,7 +2497,7 @@
       </c>
       <c r="B49" s="6">
         <f>COUNTA(Signals!B5:B2000)</f>
-        <v>787</v>
+        <v>811</v>
       </c>
     </row>
     <row r="50" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2515,7 +2515,7 @@
       </c>
       <c r="B51" s="5">
         <f>B50/B49</f>
-        <v>0.8475222363405337</v>
+        <v>0.82244143033292227</v>
       </c>
     </row>
     <row r="52" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2547,16 +2547,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A48:E48"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A11:E11"/>
+    <mergeCell ref="A47:E47"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A22:E22"/>
     <mergeCell ref="A40:E40"/>
     <mergeCell ref="A30:E30"/>
     <mergeCell ref="A29:E29"/>
     <mergeCell ref="A4:E4"/>
-    <mergeCell ref="A48:E48"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A11:E11"/>
-    <mergeCell ref="A47:E47"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -2584,40 +2584,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="99" t="s">
+      <c r="A1" s="94" t="s">
         <v>79</v>
       </c>
-      <c r="B1" s="100"/>
-      <c r="C1" s="100"/>
-      <c r="D1" s="100"/>
-      <c r="E1" s="100"/>
-      <c r="F1" s="100"/>
-      <c r="G1" s="100"/>
-      <c r="H1" s="100"/>
-      <c r="I1" s="100"/>
-      <c r="J1" s="100"/>
-      <c r="K1" s="100"/>
-      <c r="L1" s="100"/>
-      <c r="M1" s="100"/>
-      <c r="N1" s="100"/>
+      <c r="B1" s="95"/>
+      <c r="C1" s="95"/>
+      <c r="D1" s="95"/>
+      <c r="E1" s="95"/>
+      <c r="F1" s="95"/>
+      <c r="G1" s="95"/>
+      <c r="H1" s="95"/>
+      <c r="I1" s="95"/>
+      <c r="J1" s="95"/>
+      <c r="K1" s="95"/>
+      <c r="L1" s="95"/>
+      <c r="M1" s="95"/>
+      <c r="N1" s="95"/>
     </row>
     <row r="2" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="97" t="s">
+      <c r="A2" s="92" t="s">
         <v>80</v>
       </c>
-      <c r="B2" s="98"/>
-      <c r="C2" s="98"/>
-      <c r="D2" s="98"/>
-      <c r="E2" s="98"/>
-      <c r="F2" s="98"/>
-      <c r="G2" s="98"/>
-      <c r="H2" s="98"/>
-      <c r="I2" s="98"/>
-      <c r="J2" s="98"/>
-      <c r="K2" s="98"/>
-      <c r="L2" s="98"/>
-      <c r="M2" s="98"/>
-      <c r="N2" s="98"/>
+      <c r="B2" s="93"/>
+      <c r="C2" s="93"/>
+      <c r="D2" s="93"/>
+      <c r="E2" s="93"/>
+      <c r="F2" s="93"/>
+      <c r="G2" s="93"/>
+      <c r="H2" s="93"/>
+      <c r="I2" s="93"/>
+      <c r="J2" s="93"/>
+      <c r="K2" s="93"/>
+      <c r="L2" s="93"/>
+      <c r="M2" s="93"/>
+      <c r="N2" s="93"/>
     </row>
     <row r="3" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="17"/>
@@ -37999,6 +37999,27 @@
       </c>
     </row>
     <row r="792" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A792" s="12">
+        <v>46210</v>
+      </c>
+      <c r="B792" s="13" t="s">
+        <v>103</v>
+      </c>
+      <c r="C792" s="13" t="s">
+        <v>99</v>
+      </c>
+      <c r="D792" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="E792" s="14">
+        <v>0.65</v>
+      </c>
+      <c r="F792" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="G792" s="15">
+        <v>313.5</v>
+      </c>
       <c r="K792" s="26" t="str">
         <f t="shared" si="48"/>
         <v/>
@@ -38017,6 +38038,27 @@
       </c>
     </row>
     <row r="793" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A793" s="12">
+        <v>46210</v>
+      </c>
+      <c r="B793" s="13" t="s">
+        <v>112</v>
+      </c>
+      <c r="C793" s="13" t="s">
+        <v>113</v>
+      </c>
+      <c r="D793" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="E793" s="14">
+        <v>0.42</v>
+      </c>
+      <c r="F793" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="G793" s="15">
+        <v>16.39</v>
+      </c>
       <c r="K793" s="26" t="str">
         <f t="shared" si="48"/>
         <v/>
@@ -38035,6 +38077,27 @@
       </c>
     </row>
     <row r="794" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A794" s="12">
+        <v>46210</v>
+      </c>
+      <c r="B794" s="13" t="s">
+        <v>105</v>
+      </c>
+      <c r="C794" s="13" t="s">
+        <v>96</v>
+      </c>
+      <c r="D794" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="E794" s="14">
+        <v>0.47</v>
+      </c>
+      <c r="F794" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="G794" s="15">
+        <v>61.78</v>
+      </c>
       <c r="K794" s="26" t="str">
         <f t="shared" si="48"/>
         <v/>
@@ -38053,6 +38116,27 @@
       </c>
     </row>
     <row r="795" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A795" s="12">
+        <v>46210</v>
+      </c>
+      <c r="B795" s="13" t="s">
+        <v>114</v>
+      </c>
+      <c r="C795" s="13" t="s">
+        <v>113</v>
+      </c>
+      <c r="D795" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="E795" s="14">
+        <v>0.35</v>
+      </c>
+      <c r="F795" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="G795" s="15">
+        <v>175.74</v>
+      </c>
       <c r="K795" s="26" t="str">
         <f t="shared" si="48"/>
         <v/>
@@ -38071,6 +38155,27 @@
       </c>
     </row>
     <row r="796" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A796" s="12">
+        <v>46210</v>
+      </c>
+      <c r="B796" s="13" t="s">
+        <v>116</v>
+      </c>
+      <c r="C796" s="13" t="s">
+        <v>113</v>
+      </c>
+      <c r="D796" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="E796" s="14">
+        <v>0.45</v>
+      </c>
+      <c r="F796" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="G796" s="15">
+        <v>17.465</v>
+      </c>
       <c r="K796" s="26" t="str">
         <f t="shared" si="48"/>
         <v/>
@@ -38089,6 +38194,27 @@
       </c>
     </row>
     <row r="797" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A797" s="12">
+        <v>46210</v>
+      </c>
+      <c r="B797" s="13" t="s">
+        <v>104</v>
+      </c>
+      <c r="C797" s="13" t="s">
+        <v>96</v>
+      </c>
+      <c r="D797" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="E797" s="14">
+        <v>0.36</v>
+      </c>
+      <c r="F797" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="G797" s="15">
+        <v>28.035</v>
+      </c>
       <c r="K797" s="26" t="str">
         <f t="shared" si="48"/>
         <v/>
@@ -38107,6 +38233,27 @@
       </c>
     </row>
     <row r="798" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A798" s="12">
+        <v>46210</v>
+      </c>
+      <c r="B798" s="13" t="s">
+        <v>111</v>
+      </c>
+      <c r="C798" s="13" t="s">
+        <v>113</v>
+      </c>
+      <c r="D798" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="E798" s="14">
+        <v>0.6</v>
+      </c>
+      <c r="F798" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="G798" s="15">
+        <v>67.91</v>
+      </c>
       <c r="K798" s="26" t="str">
         <f t="shared" si="48"/>
         <v/>
@@ -38125,6 +38272,27 @@
       </c>
     </row>
     <row r="799" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A799" s="12">
+        <v>46210</v>
+      </c>
+      <c r="B799" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="C799" s="13" t="s">
+        <v>96</v>
+      </c>
+      <c r="D799" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="E799" s="14">
+        <v>0.52</v>
+      </c>
+      <c r="F799" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="G799" s="15">
+        <v>76.295000000000002</v>
+      </c>
       <c r="K799" s="26" t="str">
         <f t="shared" si="48"/>
         <v/>
@@ -38143,6 +38311,27 @@
       </c>
     </row>
     <row r="800" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A800" s="12">
+        <v>46210</v>
+      </c>
+      <c r="B800" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="C800" s="13" t="s">
+        <v>99</v>
+      </c>
+      <c r="D800" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="E800" s="14">
+        <v>0.65</v>
+      </c>
+      <c r="F800" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="G800" s="15">
+        <v>338.61500000000001</v>
+      </c>
       <c r="K800" s="26" t="str">
         <f t="shared" si="48"/>
         <v/>
@@ -38160,7 +38349,28 @@
         <v/>
       </c>
     </row>
-    <row r="801" spans="11:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="801" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A801" s="12">
+        <v>46210</v>
+      </c>
+      <c r="B801" s="13" t="s">
+        <v>100</v>
+      </c>
+      <c r="C801" s="13" t="s">
+        <v>96</v>
+      </c>
+      <c r="D801" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="E801" s="14">
+        <v>0.56999999999999995</v>
+      </c>
+      <c r="F801" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="G801" s="15">
+        <v>393.35</v>
+      </c>
       <c r="K801" s="26" t="str">
         <f t="shared" si="48"/>
         <v/>
@@ -38178,7 +38388,28 @@
         <v/>
       </c>
     </row>
-    <row r="802" spans="11:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="802" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A802" s="12">
+        <v>46210</v>
+      </c>
+      <c r="B802" s="13" t="s">
+        <v>101</v>
+      </c>
+      <c r="C802" s="13" t="s">
+        <v>99</v>
+      </c>
+      <c r="D802" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="E802" s="14">
+        <v>0.54</v>
+      </c>
+      <c r="F802" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="G802" s="15">
+        <v>43.21</v>
+      </c>
       <c r="K802" s="26" t="str">
         <f t="shared" si="48"/>
         <v/>
@@ -38196,7 +38427,28 @@
         <v/>
       </c>
     </row>
-    <row r="803" spans="11:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="803" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A803" s="12">
+        <v>46210</v>
+      </c>
+      <c r="B803" s="13" t="s">
+        <v>98</v>
+      </c>
+      <c r="C803" s="13" t="s">
+        <v>96</v>
+      </c>
+      <c r="D803" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="E803" s="14">
+        <v>0.62</v>
+      </c>
+      <c r="F803" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="G803" s="15">
+        <v>65.224999999999994</v>
+      </c>
       <c r="K803" s="26" t="str">
         <f t="shared" si="48"/>
         <v/>
@@ -38214,7 +38466,28 @@
         <v/>
       </c>
     </row>
-    <row r="804" spans="11:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="804" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A804" s="12">
+        <v>46210</v>
+      </c>
+      <c r="B804" s="13" t="s">
+        <v>110</v>
+      </c>
+      <c r="C804" s="13" t="s">
+        <v>99</v>
+      </c>
+      <c r="D804" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="E804" s="14">
+        <v>0.68</v>
+      </c>
+      <c r="F804" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="G804" s="15">
+        <v>188.08500000000001</v>
+      </c>
       <c r="K804" s="26" t="str">
         <f t="shared" si="48"/>
         <v/>
@@ -38232,7 +38505,28 @@
         <v/>
       </c>
     </row>
-    <row r="805" spans="11:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="805" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A805" s="12">
+        <v>46210</v>
+      </c>
+      <c r="B805" s="13" t="s">
+        <v>108</v>
+      </c>
+      <c r="C805" s="13" t="s">
+        <v>99</v>
+      </c>
+      <c r="D805" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="E805" s="14">
+        <v>0.47</v>
+      </c>
+      <c r="F805" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="G805" s="15">
+        <v>646.69000000000005</v>
+      </c>
       <c r="K805" s="26" t="str">
         <f t="shared" si="48"/>
         <v/>
@@ -38250,7 +38544,28 @@
         <v/>
       </c>
     </row>
-    <row r="806" spans="11:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="806" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A806" s="12">
+        <v>46210</v>
+      </c>
+      <c r="B806" s="13" t="s">
+        <v>115</v>
+      </c>
+      <c r="C806" s="13" t="s">
+        <v>113</v>
+      </c>
+      <c r="D806" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="E806" s="14">
+        <v>0.65</v>
+      </c>
+      <c r="F806" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="G806" s="15">
+        <v>201.69</v>
+      </c>
       <c r="K806" s="26" t="str">
         <f t="shared" si="48"/>
         <v/>
@@ -38268,7 +38583,28 @@
         <v/>
       </c>
     </row>
-    <row r="807" spans="11:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="807" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A807" s="12">
+        <v>46210</v>
+      </c>
+      <c r="B807" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="C807" s="13" t="s">
+        <v>99</v>
+      </c>
+      <c r="D807" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="E807" s="14">
+        <v>0.67</v>
+      </c>
+      <c r="F807" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="G807" s="15">
+        <v>32.579900000000002</v>
+      </c>
       <c r="K807" s="26" t="str">
         <f t="shared" si="48"/>
         <v/>
@@ -38286,7 +38622,28 @@
         <v/>
       </c>
     </row>
-    <row r="808" spans="11:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="808" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A808" s="12">
+        <v>46210</v>
+      </c>
+      <c r="B808" s="13" t="s">
+        <v>117</v>
+      </c>
+      <c r="C808" s="13" t="s">
+        <v>113</v>
+      </c>
+      <c r="D808" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="E808" s="14">
+        <v>0.4</v>
+      </c>
+      <c r="F808" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="G808" s="15">
+        <v>4.7</v>
+      </c>
       <c r="K808" s="26" t="str">
         <f t="shared" si="48"/>
         <v/>
@@ -38304,7 +38661,28 @@
         <v/>
       </c>
     </row>
-    <row r="809" spans="11:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="809" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A809" s="12">
+        <v>46210</v>
+      </c>
+      <c r="B809" s="13" t="s">
+        <v>95</v>
+      </c>
+      <c r="C809" s="13" t="s">
+        <v>96</v>
+      </c>
+      <c r="D809" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="E809" s="14">
+        <v>0.45</v>
+      </c>
+      <c r="F809" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="G809" s="15">
+        <v>111.98</v>
+      </c>
       <c r="K809" s="26" t="str">
         <f t="shared" si="48"/>
         <v/>
@@ -38322,7 +38700,28 @@
         <v/>
       </c>
     </row>
-    <row r="810" spans="11:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="810" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A810" s="12">
+        <v>46210</v>
+      </c>
+      <c r="B810" s="13" t="s">
+        <v>109</v>
+      </c>
+      <c r="C810" s="13" t="s">
+        <v>99</v>
+      </c>
+      <c r="D810" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="E810" s="14">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="F810" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="G810" s="15">
+        <v>46.024999999999999</v>
+      </c>
       <c r="K810" s="26" t="str">
         <f t="shared" si="48"/>
         <v/>
@@ -38340,7 +38739,28 @@
         <v/>
       </c>
     </row>
-    <row r="811" spans="11:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="811" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A811" s="12">
+        <v>46210</v>
+      </c>
+      <c r="B811" s="13" t="s">
+        <v>118</v>
+      </c>
+      <c r="C811" s="13" t="s">
+        <v>119</v>
+      </c>
+      <c r="D811" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="E811" s="14">
+        <v>0.54</v>
+      </c>
+      <c r="F811" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="G811" s="15">
+        <v>746.12</v>
+      </c>
       <c r="K811" s="26" t="str">
         <f t="shared" si="48"/>
         <v/>
@@ -38358,7 +38778,28 @@
         <v/>
       </c>
     </row>
-    <row r="812" spans="11:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="812" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A812" s="12">
+        <v>46210</v>
+      </c>
+      <c r="B812" s="13" t="s">
+        <v>120</v>
+      </c>
+      <c r="C812" s="13" t="s">
+        <v>119</v>
+      </c>
+      <c r="D812" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="E812" s="14">
+        <v>0.45</v>
+      </c>
+      <c r="F812" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="G812" s="15">
+        <v>707.11</v>
+      </c>
       <c r="K812" s="26" t="str">
         <f t="shared" si="48"/>
         <v/>
@@ -38376,7 +38817,28 @@
         <v/>
       </c>
     </row>
-    <row r="813" spans="11:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="813" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A813" s="12">
+        <v>46210</v>
+      </c>
+      <c r="B813" s="13" t="s">
+        <v>121</v>
+      </c>
+      <c r="C813" s="13" t="s">
+        <v>119</v>
+      </c>
+      <c r="D813" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="E813" s="14">
+        <v>0.6</v>
+      </c>
+      <c r="F813" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="G813" s="15">
+        <v>369.06</v>
+      </c>
       <c r="K813" s="26" t="str">
         <f t="shared" si="48"/>
         <v/>
@@ -38394,7 +38856,28 @@
         <v/>
       </c>
     </row>
-    <row r="814" spans="11:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="814" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A814" s="12">
+        <v>46210</v>
+      </c>
+      <c r="B814" s="13" t="s">
+        <v>122</v>
+      </c>
+      <c r="C814" s="13" t="s">
+        <v>119</v>
+      </c>
+      <c r="D814" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="E814" s="14">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="F814" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="G814" s="15">
+        <v>192.67</v>
+      </c>
       <c r="K814" s="26" t="str">
         <f t="shared" si="48"/>
         <v/>
@@ -38412,7 +38895,28 @@
         <v/>
       </c>
     </row>
-    <row r="815" spans="11:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="815" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A815" s="12">
+        <v>46210</v>
+      </c>
+      <c r="B815" s="13" t="s">
+        <v>123</v>
+      </c>
+      <c r="C815" s="13" t="s">
+        <v>119</v>
+      </c>
+      <c r="D815" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="E815" s="14">
+        <v>0.52</v>
+      </c>
+      <c r="F815" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="G815" s="15">
+        <v>380.28</v>
+      </c>
       <c r="K815" s="26" t="str">
         <f t="shared" si="48"/>
         <v/>
@@ -38430,7 +38934,7 @@
         <v/>
       </c>
     </row>
-    <row r="816" spans="11:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="816" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="K816" s="26" t="str">
         <f t="shared" si="48"/>
         <v/>
@@ -67131,43 +67635,43 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="96" t="s">
+      <c r="A1" s="99" t="s">
         <v>158</v>
       </c>
-      <c r="B1" s="93"/>
-      <c r="C1" s="93"/>
-      <c r="D1" s="93"/>
-      <c r="E1" s="93"/>
-      <c r="F1" s="93"/>
-      <c r="G1" s="93"/>
-      <c r="H1" s="93"/>
-      <c r="I1" s="93"/>
+      <c r="B1" s="97"/>
+      <c r="C1" s="97"/>
+      <c r="D1" s="97"/>
+      <c r="E1" s="97"/>
+      <c r="F1" s="97"/>
+      <c r="G1" s="97"/>
+      <c r="H1" s="97"/>
+      <c r="I1" s="97"/>
     </row>
     <row r="2" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="104" t="s">
+      <c r="A2" s="105" t="s">
         <v>159</v>
       </c>
-      <c r="B2" s="93"/>
-      <c r="C2" s="93"/>
-      <c r="D2" s="93"/>
-      <c r="E2" s="93"/>
-      <c r="F2" s="93"/>
-      <c r="G2" s="93"/>
-      <c r="H2" s="93"/>
-      <c r="I2" s="93"/>
+      <c r="B2" s="97"/>
+      <c r="C2" s="97"/>
+      <c r="D2" s="97"/>
+      <c r="E2" s="97"/>
+      <c r="F2" s="97"/>
+      <c r="G2" s="97"/>
+      <c r="H2" s="97"/>
+      <c r="I2" s="97"/>
     </row>
     <row r="4" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="105" t="s">
+      <c r="A4" s="100" t="s">
         <v>160</v>
       </c>
-      <c r="B4" s="93"/>
-      <c r="C4" s="93"/>
-      <c r="D4" s="93"/>
-      <c r="E4" s="93"/>
-      <c r="F4" s="93"/>
-      <c r="G4" s="93"/>
-      <c r="H4" s="93"/>
-      <c r="I4" s="93"/>
+      <c r="B4" s="97"/>
+      <c r="C4" s="97"/>
+      <c r="D4" s="97"/>
+      <c r="E4" s="97"/>
+      <c r="F4" s="97"/>
+      <c r="G4" s="97"/>
+      <c r="H4" s="97"/>
+      <c r="I4" s="97"/>
     </row>
     <row r="5" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="35" t="s">
@@ -67933,7 +68437,7 @@
     <row r="27" spans="1:9" ht="45" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="28" spans="1:9" ht="60" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="29" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="101" t="s">
+      <c r="A29" s="104" t="s">
         <v>190</v>
       </c>
       <c r="B29" s="102"/>
@@ -68016,7 +68520,7 @@
     <row r="34" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="35" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="36" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="101" t="s">
+      <c r="A36" s="104" t="s">
         <v>192</v>
       </c>
       <c r="B36" s="102"/>
@@ -68184,17 +68688,17 @@
       <c r="I48" s="45"/>
     </row>
     <row r="51" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="105" t="s">
+      <c r="A51" s="100" t="s">
         <v>203</v>
       </c>
-      <c r="B51" s="93"/>
-      <c r="C51" s="93"/>
-      <c r="D51" s="93"/>
-      <c r="E51" s="93"/>
-      <c r="F51" s="93"/>
-      <c r="G51" s="93"/>
-      <c r="H51" s="93"/>
-      <c r="I51" s="93"/>
+      <c r="B51" s="97"/>
+      <c r="C51" s="97"/>
+      <c r="D51" s="97"/>
+      <c r="E51" s="97"/>
+      <c r="F51" s="97"/>
+      <c r="G51" s="97"/>
+      <c r="H51" s="97"/>
+      <c r="I51" s="97"/>
     </row>
     <row r="52" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="35" t="s">
@@ -69719,7 +70223,7 @@
       </c>
     </row>
     <row r="96" spans="1:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A96" s="106" t="s">
+      <c r="A96" s="101" t="s">
         <v>245</v>
       </c>
       <c r="B96" s="102"/>
@@ -69733,13 +70237,13 @@
     </row>
   </sheetData>
   <mergeCells count="7">
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A4:I4"/>
     <mergeCell ref="A96:I96"/>
     <mergeCell ref="A29:I29"/>
     <mergeCell ref="A2:I2"/>
     <mergeCell ref="A51:I51"/>
     <mergeCell ref="A36:I36"/>
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A4:I4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -69756,10 +70260,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="96" t="s">
+      <c r="A1" s="99" t="s">
         <v>246</v>
       </c>
-      <c r="B1" s="93"/>
+      <c r="B1" s="97"/>
     </row>
     <row r="2" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3"/>
@@ -69778,10 +70282,10 @@
       <c r="B4" s="46"/>
     </row>
     <row r="5" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="95" t="s">
+      <c r="A5" s="98" t="s">
         <v>249</v>
       </c>
-      <c r="B5" s="93"/>
+      <c r="B5" s="97"/>
     </row>
     <row r="6" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
@@ -69828,10 +70332,10 @@
       <c r="B11" s="46"/>
     </row>
     <row r="12" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="95" t="s">
+      <c r="A12" s="98" t="s">
         <v>260</v>
       </c>
-      <c r="B12" s="93"/>
+      <c r="B12" s="97"/>
     </row>
     <row r="13" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
@@ -69870,10 +70374,10 @@
       <c r="B17" s="46"/>
     </row>
     <row r="18" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="95" t="s">
+      <c r="A18" s="98" t="s">
         <v>269</v>
       </c>
-      <c r="B18" s="93"/>
+      <c r="B18" s="97"/>
     </row>
     <row r="19" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
@@ -69904,10 +70408,10 @@
       <c r="B22" s="46"/>
     </row>
     <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="95" t="s">
+      <c r="A23" s="98" t="s">
         <v>276</v>
       </c>
-      <c r="B23" s="93"/>
+      <c r="B23" s="97"/>
     </row>
     <row r="24" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
@@ -69962,10 +70466,10 @@
       <c r="B30" s="46"/>
     </row>
     <row r="31" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="95" t="s">
+      <c r="A31" s="98" t="s">
         <v>289</v>
       </c>
-      <c r="B31" s="93"/>
+      <c r="B31" s="97"/>
     </row>
     <row r="32" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
@@ -70718,17 +71222,17 @@
       </c>
     </row>
     <row r="2" spans="1:9" ht="54" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="92" t="s">
+      <c r="A2" s="106" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="93"/>
-      <c r="C2" s="93"/>
-      <c r="D2" s="93"/>
-      <c r="E2" s="93"/>
-      <c r="F2" s="93"/>
-      <c r="G2" s="93"/>
-      <c r="H2" s="93"/>
-      <c r="I2" s="93"/>
+      <c r="B2" s="97"/>
+      <c r="C2" s="97"/>
+      <c r="D2" s="97"/>
+      <c r="E2" s="97"/>
+      <c r="F2" s="97"/>
+      <c r="G2" s="97"/>
+      <c r="H2" s="97"/>
+      <c r="I2" s="97"/>
     </row>
     <row r="4" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="84" t="s">

</xml_diff>